<commit_message>
Add Homework2 file to pre-week-2 folder
</commit_message>
<xml_diff>
--- a/pre-week-2/Homework2.xlsx
+++ b/pre-week-2/Homework2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\DataAnalytics-2026\pre-week-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E8A3FD0-2490-452A-BABC-6803DC19FCC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB7BE6B6-32FB-47C7-BC90-68DD50A85A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="3960" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{2937E4C4-F031-4A38-8B7A-F616A49C2F34}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2937E4C4-F031-4A38-8B7A-F616A49C2F34}"/>
   </bookViews>
   <sheets>
     <sheet name="Store_Data" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="22" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -221,7 +221,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
@@ -230,7 +230,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -280,8 +279,8 @@
             <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="dk1">
-                  <a:lumMod val="75000"/>
-                  <a:lumOff val="25000"/>
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -294,48 +293,9 @@
       </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
-    <c:view3D>
-      <c:rotX val="50"/>
-      <c:rotY val="0"/>
-      <c:depthPercent val="100"/>
-      <c:rAngAx val="0"/>
-    </c:view3D>
-    <c:floor>
-      <c:thickness val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-        <a:sp3d/>
-      </c:spPr>
-    </c:floor>
-    <c:sideWall>
-      <c:thickness val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-        <a:sp3d/>
-      </c:spPr>
-    </c:sideWall>
-    <c:backWall>
-      <c:thickness val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-        <a:sp3d/>
-      </c:spPr>
-    </c:backWall>
     <c:plotArea>
       <c:layout/>
-      <c:pie3DChart>
+      <c:pieChart>
         <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
@@ -362,13 +322,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -382,13 +341,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -402,13 +360,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -422,13 +379,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -442,13 +398,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -462,13 +417,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -484,13 +438,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -506,13 +459,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -528,13 +480,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -550,13 +501,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -572,13 +522,12 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -594,41 +543,21 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst>
-                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
                   <a:prstClr val="black">
-                    <a:alpha val="20000"/>
+                    <a:alpha val="25000"/>
                   </a:prstClr>
                 </a:outerShdw>
               </a:effectLst>
-              <a:sp3d/>
             </c:spPr>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
-              <a:pattFill prst="pct75">
-                <a:fgClr>
-                  <a:schemeClr val="dk1">
-                    <a:lumMod val="75000"/>
-                    <a:lumOff val="25000"/>
-                  </a:schemeClr>
-                </a:fgClr>
-                <a:bgClr>
-                  <a:schemeClr val="dk1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:bgClr>
-              </a:pattFill>
+              <a:noFill/>
               <a:ln>
                 <a:noFill/>
               </a:ln>
-              <a:effectLst>
-                <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:prstClr val="black">
-                    <a:alpha val="40000"/>
-                  </a:prstClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:effectLst/>
             </c:spPr>
             <c:txPr>
               <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
@@ -637,7 +566,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="lt1"/>
                     </a:solidFill>
@@ -649,7 +578,7 @@
                 <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
-            <c:dLblPos val="ctr"/>
+            <c:dLblPos val="inEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -659,13 +588,14 @@
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
-                <a:ln w="9525">
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
                   <a:solidFill>
                     <a:schemeClr val="dk1">
-                      <a:lumMod val="50000"/>
-                      <a:lumOff val="50000"/>
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
                     </a:schemeClr>
                   </a:solidFill>
+                  <a:round/>
                 </a:ln>
                 <a:effectLst/>
               </c:spPr>
@@ -676,7 +606,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Store_Data!$A$2:$C$13</c:f>
+              <c:f>Store_Data!$B$2:$C$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -755,44 +685,6 @@
                     <c:v>West</c:v>
                   </c:pt>
                 </c:lvl>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>Store A</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>Store B</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Store C</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Store D</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>Store E</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>Store F</c:v>
-                  </c:pt>
-                  <c:pt idx="6">
-                    <c:v>Store G</c:v>
-                  </c:pt>
-                  <c:pt idx="7">
-                    <c:v>Store H</c:v>
-                  </c:pt>
-                  <c:pt idx="8">
-                    <c:v>Store I</c:v>
-                  </c:pt>
-                  <c:pt idx="9">
-                    <c:v>Store J</c:v>
-                  </c:pt>
-                  <c:pt idx="10">
-                    <c:v>Store K</c:v>
-                  </c:pt>
-                  <c:pt idx="11">
-                    <c:v>Store L</c:v>
-                  </c:pt>
-                </c:lvl>
               </c:multiLvlStrCache>
             </c:multiLvlStrRef>
           </c:cat>
@@ -843,12 +735,12 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2913-47B3-AF6A-60D4F6B2F22D}"/>
+              <c16:uniqueId val="{00000000-5292-4F5A-94E2-43D9C9D0558E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="ctr"/>
+          <c:dLblPos val="inEnd"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -857,7 +749,8 @@
           <c:showBubbleSize val="0"/>
           <c:showLeaderLines val="1"/>
         </c:dLbls>
-      </c:pie3DChart>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -867,13 +760,12 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="b"/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:solidFill>
           <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="39000"/>
+            <a:alpha val="78000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:ln>
@@ -889,8 +781,8 @@
             <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="dk1">
-                  <a:lumMod val="75000"/>
-                  <a:lumOff val="25000"/>
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -914,30 +806,21 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:gradFill flip="none" rotWithShape="1">
-      <a:gsLst>
-        <a:gs pos="0">
-          <a:schemeClr val="lt1"/>
-        </a:gs>
-        <a:gs pos="39000">
-          <a:schemeClr val="lt1"/>
-        </a:gs>
-        <a:gs pos="100000">
-          <a:schemeClr val="lt1">
-            <a:lumMod val="75000"/>
-          </a:schemeClr>
-        </a:gs>
-      </a:gsLst>
-      <a:path path="circle">
-        <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-      </a:path>
-      <a:tileRect/>
-    </a:gradFill>
+    <a:pattFill prst="dkDnDiag">
+      <a:fgClr>
+        <a:schemeClr val="lt1">
+          <a:lumMod val="95000"/>
+        </a:schemeClr>
+      </a:fgClr>
+      <a:bgClr>
+        <a:schemeClr val="lt1"/>
+      </a:bgClr>
+    </a:pattFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="25000"/>
-          <a:lumOff val="75000"/>
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:round/>
@@ -1003,18 +886,18 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="264">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="261">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -1022,22 +905,11 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200" cap="all" baseline="0"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
   <cs:chartArea>
     <cs:lnRef idx="0"/>
@@ -1047,30 +919,21 @@
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:gradFill flip="none" rotWithShape="1">
-        <a:gsLst>
-          <a:gs pos="0">
-            <a:schemeClr val="lt1"/>
-          </a:gs>
-          <a:gs pos="39000">
-            <a:schemeClr val="lt1"/>
-          </a:gs>
-          <a:gs pos="100000">
-            <a:schemeClr val="lt1">
-              <a:lumMod val="75000"/>
-            </a:schemeClr>
-          </a:gs>
-        </a:gsLst>
-        <a:path path="circle">
-          <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-        </a:path>
-        <a:tileRect/>
-      </a:gradFill>
+      <a:pattFill prst="dkDnDiag">
+        <a:fgClr>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="lt1"/>
+        </a:bgClr>
+      </a:pattFill>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1085,62 +948,34 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="lt1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="pct75">
-        <a:fgClr>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
-          <a:prstClr val="black">
-            <a:alpha val="40000"/>
-          </a:prstClr>
-        </a:outerShdw>
-      </a:effectLst>
-    </cs:spPr>
-    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+    <cs:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
   </cs:dataLabel>
   <cs:dataLabelCallout>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:pattFill prst="pct75">
-        <a:fgClr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:alpha val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
           <a:schemeClr val="dk1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
           </a:schemeClr>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
-          <a:prstClr val="black">
-            <a:alpha val="40000"/>
-          </a:prstClr>
-        </a:outerShdw>
-      </a:effectLst>
+        </a:solidFill>
+      </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+    <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
       <a:spAutoFit/>
     </cs:bodyPr>
@@ -1159,9 +994,9 @@
         <a:schemeClr val="phClr"/>
       </a:solidFill>
       <a:effectLst>
-        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+        <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
           <a:prstClr val="black">
-            <a:alpha val="20000"/>
+            <a:alpha val="25000"/>
           </a:prstClr>
         </a:outerShdw>
       </a:effectLst>
@@ -1181,12 +1016,17 @@
         <a:schemeClr val="phClr"/>
       </a:solidFill>
       <a:effectLst>
-        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+        <a:outerShdw blurRad="88900" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
           <a:prstClr val="black">
             <a:alpha val="20000"/>
           </a:prstClr>
         </a:outerShdw>
       </a:effectLst>
+      <a:scene3d>
+        <a:camera prst="orthographicFront"/>
+        <a:lightRig rig="threePt" dir="t"/>
+      </a:scene3d>
+      <a:sp3d prstMaterial="matte"/>
     </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
@@ -1199,11 +1039,9 @@
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="31750" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:alpha val="85000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:round/>
       </a:ln>
@@ -1220,10 +1058,13 @@
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="phClr">
-          <a:alpha val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="phClr"/>
       </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
   <cs:dataPointMarkerLayout symbol="circle" size="6"/>
@@ -1251,62 +1092,65 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="dk1">
             <a:lumMod val="35000"/>
             <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="50000"/>
-          <a:lumOff val="50000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -1318,7 +1162,7 @@
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="dk1">
             <a:lumMod val="65000"/>
@@ -1336,6 +1180,12 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
@@ -1346,24 +1196,12 @@
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="100000">
-              <a:schemeClr val="dk1">
-                <a:lumMod val="95000"/>
-                <a:lumOff val="5000"/>
-                <a:alpha val="42000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="0">
-              <a:schemeClr val="lt1">
-                <a:lumMod val="75000"/>
-                <a:alpha val="36000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
@@ -1376,125 +1214,18 @@
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="100000">
-              <a:schemeClr val="dk1">
-                <a:lumMod val="95000"/>
-                <a:lumOff val="5000"/>
-                <a:alpha val="42000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="0">
-              <a:schemeClr val="lt1">
-                <a:lumMod val="75000"/>
-                <a:alpha val="36000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1">
-          <a:lumMod val="95000"/>
-          <a:alpha val="39000"/>
-        </a:schemeClr>
-      </a:solidFill>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
@@ -1502,7 +1233,7 @@
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="dk1">
             <a:lumMod val="50000"/>
@@ -1512,6 +1243,91 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:alpha val="78000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
   </cs:seriesLine>
   <cs:title>
     <cs:lnRef idx="0"/>
@@ -1519,8 +1335,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="1800" b="1" kern="1200" baseline="0"/>
@@ -1539,6 +1355,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:prstDash val="sysDash"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -1548,8 +1365,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1565,13 +1382,14 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="dk1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -1581,15 +1399,10 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -1694,23 +1507,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>121921</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>481012</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>483871</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>110490</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>128587</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
+        <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0BBD2FE-59D7-1A7C-D373-58F2D83AD720}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D03B01E4-5498-C429-BC9B-7E828CF37A86}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2005,7 +1818,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8C6B270E-D9B6-4E2D-9685-6945F0C3CA3E}" name="PivotTable4" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8C6B270E-D9B6-4E2D-9685-6945F0C3CA3E}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="V3:W7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -2056,7 +1869,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DB9CB7A-57A1-4779-879C-8525E47B64A2}" name="PivotTable1" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DB9CB7A-57A1-4779-879C-8525E47B64A2}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L3:M8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -2515,13 +2328,13 @@
       <c r="L4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4">
         <v>47</v>
       </c>
       <c r="V4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4">
         <v>216</v>
       </c>
     </row>
@@ -2541,13 +2354,13 @@
       <c r="L5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5">
         <v>56.666666666666664</v>
       </c>
       <c r="V5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="W5" s="6">
+      <c r="W5">
         <v>190</v>
       </c>
     </row>
@@ -2567,13 +2380,13 @@
       <c r="L6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6">
         <v>48.666666666666664</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="W6" s="6">
+      <c r="W6">
         <v>187</v>
       </c>
     </row>
@@ -2593,13 +2406,13 @@
       <c r="L7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7">
         <v>45.333333333333336</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="W7" s="6">
+      <c r="W7">
         <v>593</v>
       </c>
     </row>
@@ -2619,7 +2432,7 @@
       <c r="L8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8">
         <v>49.416666666666664</v>
       </c>
     </row>

</xml_diff>